<commit_message>
AML (マウスレイヤー) を Ctrl / Shift / Win / Alt で解除する (#28)
ryo-aoki-pc/zmk-config-LisM#22 と同じ内容 (LisM 基準)。

- excluded-positions を D / K (&mo SCRL、12 / 19) だけにする。修飾キーの位置
  (A / - / Z / / / Win / Alt) を押すと AML が切れる
- MOUSE_MOVE の修飾キーの位置を &trans にする (BASE と同じ &mt / &kp。タップで文字、
  長押しで修飾キー)
- MOUSE_SCROLL の修飾キーはそのまま。修飾キーとクリック・ホイールを組み合わせるときは
  D / K を押してから修飾キーを押す (例: D → Z → F で Shift + クリック)
- KEYMAP.html / KEYMAP.xlsx を作り直す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFG6t92cGtjhGTDoN62Yvg
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -5388,7 +5388,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -5455,7 +5455,7 @@
       <c r="N97" s="7" t="inlineStr">
         <is>
           <t>pos 21
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>LCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -5491,7 +5491,7 @@
       <c r="M98" s="9" t="inlineStr"/>
       <c r="N98" s="9" t="inlineStr">
         <is>
-          <t>RCtrl</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 22
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -5571,7 +5571,7 @@
       <c r="N99" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>LShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -5599,7 +5599,7 @@
       <c r="M100" s="9" t="inlineStr"/>
       <c r="N100" s="9" t="inlineStr">
         <is>
-          <t>RShift</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5618,13 +5618,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 35
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 36
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -5677,12 +5677,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>LWin</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>LAlt</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>
@@ -11072,7 +11072,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -11139,7 +11139,7 @@
       <c r="N97" s="7" t="inlineStr">
         <is>
           <t>pos 21
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -11151,7 +11151,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -11175,7 +11175,7 @@
       <c r="M98" s="9" t="inlineStr"/>
       <c r="N98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RCTRL</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -11188,7 +11188,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 22
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -11255,7 +11255,7 @@
       <c r="N99" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -11283,7 +11283,7 @@
       <c r="M100" s="9" t="inlineStr"/>
       <c r="N100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RIGHT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -11302,13 +11302,13 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 35
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 36
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -11361,12 +11361,12 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_WIN</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_ALT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr"/>

</xml_diff>